<commit_message>
refactor: update app and excel handlers, add v2 sample
</commit_message>
<xml_diff>
--- a/samples/Pranay_HOME_E-Bill_Analysis_FILLED.xlsx
+++ b/samples/Pranay_HOME_E-Bill_Analysis_FILLED.xlsx
@@ -682,10 +682,8 @@
           <t>Consumer No</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
-        <is>
-          <t>439320095567</t>
-        </is>
+      <c r="D2" s="8" t="n">
+        <v>439320095567</v>
       </c>
       <c r="E2" s="9" t="n"/>
       <c r="F2" s="10" t="n"/>

</xml_diff>